<commit_message>
Arreglo de cvs a xlsx
</commit_message>
<xml_diff>
--- a/data/SPR_BS_master.xlsx
+++ b/data/SPR_BS_master.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\SPR-BS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88742377-E2DD-4382-96A4-A188F83AEBB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E71999E-D957-4068-AD67-3AC30AF397CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="master_bono" sheetId="1" r:id="rId1"/>
     <sheet name="README" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -492,7 +492,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -519,9 +519,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2681,7 +2678,7 @@
       </c>
     </row>
     <row r="58" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2873,7 +2870,7 @@
       </c>
     </row>
     <row r="64" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="10" t="s">
+      <c r="A64" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B64" s="7" t="s">

</xml_diff>

<commit_message>
Adicion de LECAPS y BONCAPS
</commit_message>
<xml_diff>
--- a/data/SPR_BS_master.xlsx
+++ b/data/SPR_BS_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomas\SPR-BS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E71999E-D957-4068-AD67-3AC30AF397CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9928067-7160-4DEE-89B9-8B8787C7083D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="140">
   <si>
     <t>codigo</t>
   </si>
@@ -406,6 +406,57 @@
   </si>
   <si>
     <t>SOBERANO</t>
+  </si>
+  <si>
+    <t>S27F6</t>
+  </si>
+  <si>
+    <t>LECAP</t>
+  </si>
+  <si>
+    <t>S17A6</t>
+  </si>
+  <si>
+    <t>S16M6</t>
+  </si>
+  <si>
+    <t>S30A6</t>
+  </si>
+  <si>
+    <t>S29Y6</t>
+  </si>
+  <si>
+    <t>S31L6</t>
+  </si>
+  <si>
+    <t>S31G6</t>
+  </si>
+  <si>
+    <t>S30O6</t>
+  </si>
+  <si>
+    <t>S30N6</t>
+  </si>
+  <si>
+    <t>T13F6</t>
+  </si>
+  <si>
+    <t>BONCAP</t>
+  </si>
+  <si>
+    <t>T30J6</t>
+  </si>
+  <si>
+    <t>T15E7</t>
+  </si>
+  <si>
+    <t>T30A7</t>
+  </si>
+  <si>
+    <t>T31Y7</t>
+  </si>
+  <si>
+    <t>T30J7</t>
   </si>
 </sst>
 </file>
@@ -717,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1048576"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.21875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="15.33203125" style="1" customWidth="1"/>
@@ -2285,26 +2336,24 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="8" t="s">
-        <v>60</v>
+      <c r="A46" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="2">
-        <v>45296</v>
-      </c>
+      <c r="C46" s="1"/>
       <c r="D46" s="2">
-        <v>46691</v>
+        <v>46080</v>
       </c>
       <c r="E46" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H46" s="1">
         <v>100</v>
@@ -2316,30 +2365,28 @@
         <v>11</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>61</v>
+        <v>125</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C47" s="2">
-        <v>45596</v>
-      </c>
+      <c r="C47" s="1"/>
       <c r="D47" s="2">
-        <v>46691</v>
+        <v>46129</v>
       </c>
       <c r="E47" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H47" s="1">
         <v>100</v>
@@ -2351,27 +2398,28 @@
         <v>11</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>62</v>
+        <v>126</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C48" s="1"/>
       <c r="D48" s="2">
-        <v>46691</v>
+        <v>46097</v>
       </c>
       <c r="E48" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F48" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H48" s="1">
         <v>100</v>
@@ -2383,30 +2431,28 @@
         <v>11</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C49" s="2">
-        <v>45352</v>
-      </c>
+      <c r="C49" s="1"/>
       <c r="D49" s="2">
-        <v>46691</v>
+        <v>46142</v>
       </c>
       <c r="E49" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H49" s="1">
         <v>100</v>
@@ -2418,27 +2464,28 @@
         <v>11</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C50" s="1"/>
       <c r="D50" s="2">
-        <v>46691</v>
+        <v>46171</v>
       </c>
       <c r="E50" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H50" s="1">
         <v>100</v>
@@ -2447,30 +2494,31 @@
         <v>100</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>66</v>
+        <v>129</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C51" s="1"/>
       <c r="D51" s="2">
-        <v>46691</v>
+        <v>46234</v>
       </c>
       <c r="E51" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F51" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H51" s="1">
         <v>100</v>
@@ -2479,30 +2527,31 @@
         <v>100</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>67</v>
+        <v>130</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C52" s="1"/>
       <c r="D52" s="2">
-        <v>46691</v>
+        <v>46265</v>
       </c>
       <c r="E52" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F52" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H52" s="1">
         <v>100</v>
@@ -2511,30 +2560,31 @@
         <v>100</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>68</v>
+        <v>131</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C53" s="1"/>
       <c r="D53" s="2">
-        <v>46691</v>
+        <v>46325</v>
       </c>
       <c r="E53" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F53" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H53" s="1">
         <v>100</v>
@@ -2543,30 +2593,31 @@
         <v>100</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A54" s="9" t="s">
-        <v>69</v>
+      <c r="A54" s="1" t="s">
+        <v>132</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C54" s="1"/>
       <c r="D54" s="2">
-        <v>46691</v>
+        <v>46356</v>
       </c>
       <c r="E54" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F54" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H54" s="1">
         <v>100</v>
@@ -2575,30 +2626,31 @@
         <v>100</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A55" s="9" t="s">
-        <v>71</v>
+      <c r="A55" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C55" s="1"/>
       <c r="D55" s="2">
-        <v>46691</v>
+        <v>46066</v>
       </c>
       <c r="E55" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F55" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H55" s="1">
         <v>100</v>
@@ -2607,30 +2659,31 @@
         <v>100</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A56" s="9" t="s">
-        <v>72</v>
+      <c r="A56" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C56" s="1"/>
       <c r="D56" s="2">
-        <v>46691</v>
+        <v>46203</v>
       </c>
       <c r="E56" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F56" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H56" s="1">
         <v>100</v>
@@ -2639,30 +2692,31 @@
         <v>100</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A57" s="9" t="s">
-        <v>73</v>
+      <c r="A57" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C57" s="1"/>
       <c r="D57" s="2">
-        <v>46691</v>
+        <v>46402</v>
       </c>
       <c r="E57" s="3">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F57" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H57" s="1">
         <v>100</v>
@@ -2671,126 +2725,132 @@
         <v>100</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>74</v>
+        <v>137</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C58" s="1"/>
       <c r="D58" s="2">
-        <v>46173</v>
+        <v>46507</v>
       </c>
       <c r="E58" s="3">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F58" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H58" s="1">
         <v>100</v>
       </c>
       <c r="I58" s="1">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
-        <v>75</v>
+      <c r="A59" s="1" t="s">
+        <v>138</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C59" s="1"/>
       <c r="D59" s="2">
-        <v>46173</v>
+        <v>46538</v>
       </c>
       <c r="E59" s="3">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F59" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H59" s="1">
         <v>100</v>
       </c>
       <c r="I59" s="1">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>65</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C60" s="1"/>
       <c r="D60" s="2">
-        <v>46173</v>
+        <v>46568</v>
       </c>
       <c r="E60" s="3">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="F60" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H60" s="1">
         <v>100</v>
       </c>
       <c r="I60" s="1">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>77</v>
+      <c r="A61" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C61" s="2">
+        <v>45296</v>
+      </c>
       <c r="D61" s="2">
-        <v>46805</v>
+        <v>46691</v>
       </c>
       <c r="E61" s="3">
-        <v>0.35920000000000002</v>
+        <v>0.05</v>
       </c>
       <c r="F61" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H61" s="1">
         <v>100</v>
@@ -2807,16 +2867,19 @@
     </row>
     <row r="62" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="C62" s="2">
+        <v>45596</v>
       </c>
       <c r="D62" s="2">
-        <v>48397</v>
+        <v>46691</v>
       </c>
       <c r="E62" s="3">
-        <v>6.6299999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F62" s="1">
         <v>2</v>
@@ -2831,7 +2894,7 @@
         <v>100</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="K62" s="1" t="s">
         <v>122</v>
@@ -2839,16 +2902,16 @@
     </row>
     <row r="63" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D63" s="2">
-        <v>50284</v>
+        <v>46691</v>
       </c>
       <c r="E63" s="3">
-        <v>5.8799999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F63" s="1">
         <v>2</v>
@@ -2871,16 +2934,19 @@
     </row>
     <row r="64" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B64" s="7" t="s">
-        <v>18</v>
+        <v>63</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C64" s="2">
+        <v>45352</v>
       </c>
       <c r="D64" s="2">
-        <v>50284</v>
+        <v>46691</v>
       </c>
       <c r="E64" s="3">
-        <v>6.6299999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F64" s="1">
         <v>2</v>
@@ -2892,7 +2958,7 @@
         <v>100</v>
       </c>
       <c r="I64" s="1">
-        <v>91.84</v>
+        <v>100</v>
       </c>
       <c r="J64" s="1" t="s">
         <v>11</v>
@@ -2902,17 +2968,17 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="9" t="s">
-        <v>81</v>
+      <c r="A65" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D65" s="2">
-        <v>50284</v>
+        <v>46691</v>
       </c>
       <c r="E65" s="3">
-        <v>6.6299999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F65" s="1">
         <v>2</v>
@@ -2924,10 +2990,10 @@
         <v>100</v>
       </c>
       <c r="I65" s="1">
-        <v>91.84</v>
+        <v>100</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="K65" s="1" t="s">
         <v>122</v>
@@ -2935,16 +3001,16 @@
     </row>
     <row r="66" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D66" s="2">
-        <v>50284</v>
+        <v>46691</v>
       </c>
       <c r="E66" s="3">
-        <v>5.8799999999999998E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F66" s="1">
         <v>2</v>
@@ -2959,30 +3025,30 @@
         <v>100</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="K66" s="1" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A67" s="6" t="s">
-        <v>83</v>
+      <c r="A67" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D67" s="2">
-        <v>46084</v>
+        <v>46691</v>
       </c>
       <c r="E67" s="3">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="F67" s="1">
         <v>2</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H67" s="1">
         <v>100</v>
@@ -2991,30 +3057,30 @@
         <v>100</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="K67" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D68" s="2">
-        <v>46092</v>
+        <v>46691</v>
       </c>
       <c r="E68" s="3">
-        <v>7.4899999999999994E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F68" s="1">
         <v>2</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H68" s="1">
         <v>100</v>
@@ -3023,257 +3089,251 @@
         <v>100</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A69" s="6" t="s">
-        <v>85</v>
+      <c r="A69" s="9" t="s">
+        <v>69</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D69" s="2">
-        <v>46170</v>
+        <v>46691</v>
       </c>
       <c r="E69" s="3">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="F69" s="1">
+        <v>2</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H69" s="1">
+        <v>100</v>
+      </c>
+      <c r="I69" s="1">
+        <v>100</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A70" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70" s="2">
+        <v>46691</v>
+      </c>
+      <c r="E70" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="F70" s="1">
+        <v>2</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H70" s="1">
+        <v>100</v>
+      </c>
+      <c r="I70" s="1">
+        <v>100</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A71" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="2">
+        <v>46691</v>
+      </c>
+      <c r="E71" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="F71" s="1">
+        <v>2</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H71" s="1">
+        <v>100</v>
+      </c>
+      <c r="I71" s="1">
+        <v>100</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A72" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D72" s="2">
+        <v>46691</v>
+      </c>
+      <c r="E72" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="F72" s="1">
+        <v>2</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H72" s="1">
+        <v>100</v>
+      </c>
+      <c r="I72" s="1">
+        <v>100</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="2">
+        <v>46173</v>
+      </c>
+      <c r="E73" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="F73" s="1">
         <v>4</v>
       </c>
-      <c r="G69" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H69" s="1">
-        <v>100</v>
-      </c>
-      <c r="I69" s="1">
-        <v>100</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C70" s="1"/>
-      <c r="D70" s="2">
-        <v>46186</v>
-      </c>
-      <c r="E70" s="3">
-        <v>0.06</v>
-      </c>
-      <c r="F70" s="1">
+      <c r="G73" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H73" s="1">
+        <v>100</v>
+      </c>
+      <c r="I73" s="1">
+        <v>67</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A74" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D74" s="2">
+        <v>46173</v>
+      </c>
+      <c r="E74" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="F74" s="1">
         <v>4</v>
       </c>
-      <c r="G70" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H70" s="1">
-        <v>100</v>
-      </c>
-      <c r="I70" s="1">
-        <v>100</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C71" s="1"/>
-      <c r="D71" s="2">
-        <v>46348</v>
-      </c>
-      <c r="E71" s="3">
-        <v>9.7500000000000003E-2</v>
-      </c>
-      <c r="F71" s="1">
-        <v>2</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H71" s="1">
-        <v>100</v>
-      </c>
-      <c r="I71" s="1">
-        <v>100</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A72" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C72" s="1"/>
-      <c r="D72" s="2">
-        <v>46683</v>
-      </c>
-      <c r="E72" s="3">
-        <v>5.7500000000000002E-2</v>
-      </c>
-      <c r="F72" s="1">
-        <v>2</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H72" s="1">
-        <v>100</v>
-      </c>
-      <c r="I72" s="1">
-        <v>100</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C73" s="1"/>
-      <c r="D73" s="2">
-        <v>47070</v>
-      </c>
-      <c r="E73" s="3">
-        <v>6.25E-2</v>
-      </c>
-      <c r="F73" s="1">
-        <v>2</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H73" s="1">
-        <v>100</v>
-      </c>
-      <c r="I73" s="1">
-        <v>100</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C74" s="1"/>
-      <c r="D74" s="2">
-        <v>47388</v>
-      </c>
-      <c r="E74" s="3">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F74" s="1">
-        <v>2</v>
-      </c>
       <c r="G74" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H74" s="1">
         <v>100</v>
       </c>
       <c r="I74" s="1">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="75" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A75" s="6" t="s">
-        <v>91</v>
+      <c r="A75" s="1" t="s">
+        <v>76</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C75" s="1"/>
+        <v>65</v>
+      </c>
       <c r="D75" s="2">
-        <v>47414</v>
+        <v>46173</v>
       </c>
       <c r="E75" s="3">
-        <v>7.2499999999999995E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F75" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H75" s="1">
         <v>100</v>
       </c>
       <c r="I75" s="1">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="K75" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="76" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D76" s="2">
-        <v>47357</v>
+        <v>46805</v>
       </c>
       <c r="E76" s="3">
-        <v>7.4999999999999997E-2</v>
+        <v>0.35920000000000002</v>
       </c>
       <c r="F76" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G76" s="1" t="s">
         <v>20</v>
@@ -3288,27 +3348,27 @@
         <v>11</v>
       </c>
       <c r="K76" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="77" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A77" s="6" t="s">
-        <v>93</v>
+      <c r="A77" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D77" s="2">
-        <v>48131</v>
+        <v>48397</v>
       </c>
       <c r="E77" s="3">
-        <v>7.6499999999999999E-2</v>
+        <v>6.6299999999999998E-2</v>
       </c>
       <c r="F77" s="1">
         <v>2</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H77" s="1">
         <v>100</v>
@@ -3317,31 +3377,30 @@
         <v>100</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K77" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="78" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A78" s="6" t="s">
-        <v>94</v>
+      <c r="A78" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C78" s="1"/>
+        <v>11</v>
+      </c>
       <c r="D78" s="2">
-        <v>48165</v>
+        <v>50284</v>
       </c>
       <c r="E78" s="3">
-        <v>7.2499999999999995E-2</v>
+        <v>5.8799999999999998E-2</v>
       </c>
       <c r="F78" s="1">
         <v>2</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H78" s="1">
         <v>100</v>
@@ -3353,22 +3412,21 @@
         <v>11</v>
       </c>
       <c r="K78" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="79" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C79" s="1"/>
+        <v>80</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="D79" s="2">
-        <v>48727</v>
+        <v>50284</v>
       </c>
       <c r="E79" s="3">
-        <v>9.5000000000000001E-2</v>
+        <v>6.6299999999999998E-2</v>
       </c>
       <c r="F79" s="1">
         <v>2</v>
@@ -3380,100 +3438,97 @@
         <v>100</v>
       </c>
       <c r="I79" s="1">
-        <v>100</v>
+        <v>91.84</v>
       </c>
       <c r="J79" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K79" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A80" s="6" t="s">
-        <v>96</v>
+      <c r="A80" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C80" s="1"/>
       <c r="D80" s="2">
-        <v>46203</v>
+        <v>50284</v>
       </c>
       <c r="E80" s="3">
-        <v>0.1095</v>
+        <v>6.6299999999999998E-2</v>
       </c>
       <c r="F80" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H80" s="1">
         <v>100</v>
       </c>
       <c r="I80" s="1">
-        <v>100</v>
+        <v>91.84</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K80" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="81" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A81" s="6" t="s">
-        <v>97</v>
+      <c r="A81" s="1" t="s">
+        <v>82</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C81" s="1"/>
       <c r="D81" s="2">
-        <v>46221</v>
+        <v>50284</v>
       </c>
       <c r="E81" s="3">
+        <v>5.8799999999999998E-2</v>
+      </c>
+      <c r="F81" s="1">
+        <v>2</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H81" s="1">
+        <v>100</v>
+      </c>
+      <c r="I81" s="1">
+        <v>100</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D82" s="2">
+        <v>46084</v>
+      </c>
+      <c r="E82" s="3">
         <v>0.08</v>
       </c>
-      <c r="F81" s="1">
-        <v>2</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H81" s="1">
-        <v>100</v>
-      </c>
-      <c r="I81" s="1">
-        <v>100</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K81" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A82" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C82" s="1"/>
-      <c r="D82" s="2">
-        <v>46507</v>
-      </c>
-      <c r="E82" s="3">
-        <v>9.1300000000000006E-2</v>
-      </c>
       <c r="F82" s="1">
         <v>2</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H82" s="1">
         <v>100</v>
@@ -3490,17 +3545,16 @@
     </row>
     <row r="83" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C83" s="1"/>
       <c r="D83" s="2">
-        <v>47292</v>
+        <v>46092</v>
       </c>
       <c r="E83" s="3">
-        <v>0.08</v>
+        <v>7.4899999999999994E-2</v>
       </c>
       <c r="F83" s="1">
         <v>2</v>
@@ -3523,23 +3577,22 @@
     </row>
     <row r="84" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C84" s="1"/>
       <c r="D84" s="2">
-        <v>47299</v>
+        <v>46170</v>
       </c>
       <c r="E84" s="3">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="F84" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H84" s="1">
         <v>100</v>
@@ -3555,21 +3608,21 @@
       </c>
     </row>
     <row r="85" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1" t="s">
-        <v>101</v>
+      <c r="A85" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C85" s="1"/>
       <c r="D85" s="2">
-        <v>47686</v>
+        <v>46186</v>
       </c>
       <c r="E85" s="3">
-        <v>8.7499999999999994E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F85" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G85" s="1" t="s">
         <v>20</v>
@@ -3589,16 +3642,17 @@
     </row>
     <row r="86" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C86" s="1"/>
       <c r="D86" s="2">
-        <v>48047</v>
+        <v>46348</v>
       </c>
       <c r="E86" s="3">
-        <v>9.7000000000000003E-2</v>
+        <v>9.7500000000000003E-2</v>
       </c>
       <c r="F86" s="1">
         <v>2</v>
@@ -3621,23 +3675,23 @@
     </row>
     <row r="87" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C87" s="1"/>
       <c r="D87" s="2">
-        <v>48102</v>
+        <v>46683</v>
       </c>
       <c r="E87" s="3">
-        <v>8.7499999999999994E-2</v>
+        <v>5.7500000000000002E-2</v>
       </c>
       <c r="F87" s="1">
         <v>2</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H87" s="1">
         <v>100</v>
@@ -3653,17 +3707,18 @@
       </c>
     </row>
     <row r="88" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
-        <v>104</v>
+      <c r="A88" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C88" s="1"/>
       <c r="D88" s="2">
-        <v>48364</v>
+        <v>47070</v>
       </c>
       <c r="E88" s="3">
-        <v>8.5000000000000006E-2</v>
+        <v>6.25E-2</v>
       </c>
       <c r="F88" s="1">
         <v>2</v>
@@ -3686,22 +3741,23 @@
     </row>
     <row r="89" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C89" s="1"/>
       <c r="D89" s="2">
-        <v>48503</v>
+        <v>47388</v>
       </c>
       <c r="E89" s="3">
-        <v>7.8799999999999995E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F89" s="1">
         <v>2</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H89" s="1">
         <v>100</v>
@@ -3717,23 +3773,24 @@
       </c>
     </row>
     <row r="90" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
-        <v>106</v>
+      <c r="A90" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C90" s="1"/>
       <c r="D90" s="2">
-        <v>48740</v>
+        <v>47414</v>
       </c>
       <c r="E90" s="3">
-        <v>8.5000000000000006E-2</v>
+        <v>7.2499999999999995E-2</v>
       </c>
       <c r="F90" s="1">
         <v>2</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H90" s="1">
         <v>100</v>
@@ -3748,24 +3805,24 @@
         <v>121</v>
       </c>
     </row>
-    <row r="91" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="6" t="s">
-        <v>107</v>
+    <row r="91" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D91" s="2">
-        <v>48852</v>
+        <v>47357</v>
       </c>
       <c r="E91" s="3">
-        <v>7.0000000000000007E-2</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="F91" s="1">
         <v>2</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H91" s="1">
         <v>100</v>
@@ -3781,18 +3838,17 @@
       </c>
     </row>
     <row r="92" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
-        <v>108</v>
+      <c r="A92" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C92" s="1"/>
       <c r="D92" s="2">
-        <v>49399</v>
+        <v>48131</v>
       </c>
       <c r="E92" s="3">
-        <v>0.08</v>
+        <v>7.6499999999999999E-2</v>
       </c>
       <c r="F92" s="1">
         <v>2</v>
@@ -3815,17 +3871,17 @@
     </row>
     <row r="93" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C93" s="1"/>
       <c r="D93" s="2">
-        <v>49653</v>
+        <v>48165</v>
       </c>
       <c r="E93" s="3">
-        <v>7.6300000000000007E-2</v>
+        <v>7.2499999999999995E-2</v>
       </c>
       <c r="F93" s="1">
         <v>2</v>
@@ -3847,18 +3903,18 @@
       </c>
     </row>
     <row r="94" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A94" s="6" t="s">
-        <v>110</v>
+      <c r="A94" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C94" s="1"/>
       <c r="D94" s="2">
-        <v>48961</v>
+        <v>48727</v>
       </c>
       <c r="E94" s="3">
-        <v>8.7499999999999994E-2</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="F94" s="1">
         <v>2</v>
@@ -3880,57 +3936,502 @@
       </c>
     </row>
     <row r="95" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A95" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C95" s="1"/>
+      <c r="D95" s="2">
+        <v>46203</v>
+      </c>
+      <c r="E95" s="3">
+        <v>0.1095</v>
+      </c>
+      <c r="F95" s="1">
+        <v>4</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H95" s="1">
+        <v>100</v>
+      </c>
+      <c r="I95" s="1">
+        <v>100</v>
+      </c>
+      <c r="J95" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="96" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C96" s="1"/>
-    </row>
-    <row r="97" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D96" s="2">
+        <v>46221</v>
+      </c>
+      <c r="E96" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="F96" s="1">
+        <v>2</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H96" s="1">
+        <v>100</v>
+      </c>
+      <c r="I96" s="1">
+        <v>100</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C97" s="1"/>
-    </row>
-    <row r="98" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D97" s="2">
+        <v>46507</v>
+      </c>
+      <c r="E97" s="3">
+        <v>9.1300000000000006E-2</v>
+      </c>
+      <c r="F97" s="1">
+        <v>2</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H97" s="1">
+        <v>100</v>
+      </c>
+      <c r="I97" s="1">
+        <v>100</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C98" s="1"/>
-    </row>
-    <row r="99" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D98" s="2">
+        <v>47292</v>
+      </c>
+      <c r="E98" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="F98" s="1">
+        <v>2</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H98" s="1">
+        <v>100</v>
+      </c>
+      <c r="I98" s="1">
+        <v>100</v>
+      </c>
+      <c r="J98" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C99" s="1"/>
-    </row>
-    <row r="100" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D99" s="2">
+        <v>47299</v>
+      </c>
+      <c r="E99" s="3">
+        <v>0.09</v>
+      </c>
+      <c r="F99" s="1">
+        <v>2</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H99" s="1">
+        <v>100</v>
+      </c>
+      <c r="I99" s="1">
+        <v>100</v>
+      </c>
+      <c r="J99" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C100" s="1"/>
-    </row>
-    <row r="101" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C101" s="1"/>
-    </row>
-    <row r="102" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D100" s="2">
+        <v>47686</v>
+      </c>
+      <c r="E100" s="3">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="F100" s="1">
+        <v>2</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H100" s="1">
+        <v>100</v>
+      </c>
+      <c r="I100" s="1">
+        <v>100</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D101" s="2">
+        <v>48047</v>
+      </c>
+      <c r="E101" s="3">
+        <v>9.7000000000000003E-2</v>
+      </c>
+      <c r="F101" s="1">
+        <v>2</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H101" s="1">
+        <v>100</v>
+      </c>
+      <c r="I101" s="1">
+        <v>100</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A102" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C102" s="1"/>
-    </row>
-    <row r="103" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C103" s="1"/>
-    </row>
-    <row r="104" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C104" s="1"/>
-    </row>
-    <row r="105" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C105" s="1"/>
-    </row>
-    <row r="106" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="C106" s="1"/>
-    </row>
-    <row r="107" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D102" s="2">
+        <v>48102</v>
+      </c>
+      <c r="E102" s="3">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="F102" s="1">
+        <v>2</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H102" s="1">
+        <v>100</v>
+      </c>
+      <c r="I102" s="1">
+        <v>100</v>
+      </c>
+      <c r="J102" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K102" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D103" s="2">
+        <v>48364</v>
+      </c>
+      <c r="E103" s="3">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="F103" s="1">
+        <v>2</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H103" s="1">
+        <v>100</v>
+      </c>
+      <c r="I103" s="1">
+        <v>100</v>
+      </c>
+      <c r="J103" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A104" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D104" s="2">
+        <v>48503</v>
+      </c>
+      <c r="E104" s="3">
+        <v>7.8799999999999995E-2</v>
+      </c>
+      <c r="F104" s="1">
+        <v>2</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H104" s="1">
+        <v>100</v>
+      </c>
+      <c r="I104" s="1">
+        <v>100</v>
+      </c>
+      <c r="J104" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K104" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D105" s="2">
+        <v>48740</v>
+      </c>
+      <c r="E105" s="3">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="F105" s="1">
+        <v>2</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H105" s="1">
+        <v>100</v>
+      </c>
+      <c r="I105" s="1">
+        <v>100</v>
+      </c>
+      <c r="J105" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K105" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D106" s="2">
+        <v>48852</v>
+      </c>
+      <c r="E106" s="3">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F106" s="1">
+        <v>2</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H106" s="1">
+        <v>100</v>
+      </c>
+      <c r="I106" s="1">
+        <v>100</v>
+      </c>
+      <c r="J106" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K106" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C107" s="1"/>
-    </row>
-    <row r="108" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D107" s="2">
+        <v>49399</v>
+      </c>
+      <c r="E107" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="F107" s="1">
+        <v>2</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H107" s="1">
+        <v>100</v>
+      </c>
+      <c r="I107" s="1">
+        <v>100</v>
+      </c>
+      <c r="J107" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K107" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A108" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C108" s="1"/>
-    </row>
-    <row r="109" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D108" s="2">
+        <v>49653</v>
+      </c>
+      <c r="E108" s="3">
+        <v>7.6300000000000007E-2</v>
+      </c>
+      <c r="F108" s="1">
+        <v>2</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H108" s="1">
+        <v>100</v>
+      </c>
+      <c r="I108" s="1">
+        <v>100</v>
+      </c>
+      <c r="J108" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K108" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A109" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="C109" s="1"/>
-    </row>
-    <row r="110" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D109" s="2">
+        <v>48961</v>
+      </c>
+      <c r="E109" s="3">
+        <v>8.7499999999999994E-2</v>
+      </c>
+      <c r="F109" s="1">
+        <v>2</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H109" s="1">
+        <v>100</v>
+      </c>
+      <c r="I109" s="1">
+        <v>100</v>
+      </c>
+      <c r="J109" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K109" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C110" s="1"/>
     </row>
-    <row r="111" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C111" s="1"/>
     </row>
-    <row r="112" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C112" s="1"/>
     </row>
     <row r="113" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -4071,8 +4572,6 @@
     <row r="158" spans="3:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C158" s="1"/>
     </row>
-    <row r="1048575" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="1048576" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>